<commit_message>
inquired status of SNGP transmission case
</commit_message>
<xml_diff>
--- a/_generic/NewsPaperAds.xlsx
+++ b/_generic/NewsPaperAds.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="StampPaper" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="177">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -590,6 +590,21 @@
   <si>
     <t xml:space="preserve">distinctive Number corrigendum-PN
 Signature of guar1, 2 and applicant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CDCSR-LHR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNGP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAK-SNGP-2603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transmission Case - SNGPL - Late Mohammad Ayub Khan, Folio Nr: 125005252</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inquired about status of transmission case, via email</t>
   </si>
 </sst>
 </file>
@@ -686,7 +701,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -741,6 +756,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1065,7 +1084,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="11.53"/>
@@ -1521,6 +1540,13 @@
       <c r="E20" s="9" t="s">
         <v>100</v>
       </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0"/>
+      <c r="B21" s="0"/>
+      <c r="C21" s="0"/>
+      <c r="D21" s="0"/>
+      <c r="E21" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1538,7 +1564,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="7" width="11.53"/>
@@ -2101,6 +2127,33 @@
         <v>1</v>
       </c>
     </row>
+    <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="E24" s="0"/>
+      <c r="F24" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="I24" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H8" r:id="rId1" display="Mr. Khalid Pervez: khalid.pervez@js.com, via PAKPOST dispatched"/>

</xml_diff>